<commit_message>
updated excel file and Data Structure Intro feature file
</commit_message>
<xml_diff>
--- a/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
+++ b/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5BFCB8F7-ED19-43F0-8CC2-820C6282730F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{8BC72E55-6003-4232-89B1-493985A72B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
@@ -61,6 +61,9 @@
     <t>password confirmation</t>
   </si>
   <si>
+    <t>techtitanstest3</t>
+  </si>
+  <si>
     <t>#</t>
   </si>
   <si>
@@ -92,9 +95,6 @@
   </si>
   <si>
     <t>SyntaxError: bad input on line 1</t>
-  </si>
-  <si>
-    <t>techtitanstest4</t>
   </si>
 </sst>
 </file>
@@ -560,102 +560,102 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3" t="s">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="C8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="D8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="3">
+      <c r="A9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="1">
         <v>12345678901</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="1">
         <v>12345678901</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>13</v>
+      <c r="D9" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -688,10 +688,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -742,7 +742,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="1"/>
     </row>
@@ -754,10 +754,10 @@
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Latest updates for Data driven testing
</commit_message>
<xml_diff>
--- a/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
+++ b/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{07D70AB1-60BA-4C51-91CA-CBC9110F3EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{14A1762D-0F3A-47D2-B4F4-4E1BB3B8E772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
@@ -61,9 +61,6 @@
     <t>password confirmation</t>
   </si>
   <si>
-    <t>techtitanstest3</t>
-  </si>
-  <si>
     <t>#</t>
   </si>
   <si>
@@ -95,6 +92,9 @@
   </si>
   <si>
     <t>SyntaxError: bad input on line 1</t>
+  </si>
+  <si>
+    <t>techtitanstest5</t>
   </si>
 </sst>
 </file>
@@ -560,7 +560,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
@@ -569,7 +569,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -582,7 +582,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -592,7 +592,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>4</v>
@@ -604,49 +604,49 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" s="1">
         <v>12345678901</v>
@@ -655,7 +655,7 @@
         <v>12345678901</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -688,10 +688,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -742,7 +742,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1"/>
     </row>
@@ -754,10 +754,10 @@
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes in driver initialization and added extent reports and Screenshot feature
</commit_message>
<xml_diff>
--- a/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
+++ b/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{14A1762D-0F3A-47D2-B4F4-4E1BB3B8E772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{1BB46C4A-4AB7-4588-A0F4-66F53213A46A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="tryEditor" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:H23"/>
+  <oleSize ref="A1:I8"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="24">
   <si>
     <t>username</t>
   </si>
@@ -704,62 +704,35 @@
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1"/>
+      <c r="C3" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>22</v>
       </c>
     </row>
+    <row r="5" spans="1:4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:4" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated test data for Register test case
</commit_message>
<xml_diff>
--- a/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
+++ b/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{37C6522A-A047-449F-84E3-DA5168AE25AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{80BDCD6B-CFA8-4243-AF60-A3B19C85BA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="tryEditor" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:G23"/>
+  <oleSize ref="A1:H23"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -94,7 +94,7 @@
     <t>SyntaxError: bad input on line 1</t>
   </si>
   <si>
-    <t>techtitanstest5</t>
+    <t>techtitanstest07</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updated test data for new user registration test case
</commit_message>
<xml_diff>
--- a/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
+++ b/DSAlgoPortal/src/test/resources/ExcelTestData/LoginData.xlsx
@@ -3,7 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{80BDCD6B-CFA8-4243-AF60-A3B19C85BA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manal_\git\DSAlgoTechTitans\DSAlgoPortal\src\test\resources\ExcelTestData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4689C83B-D8DD-4554-B0F4-B70D5467CB3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,7 +18,6 @@
     <sheet name="tryEditor" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:H23"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -94,7 +98,7 @@
     <t>SyntaxError: bad input on line 1</t>
   </si>
   <si>
-    <t>techtitanstest07</t>
+    <t>techtitanstest08</t>
   </si>
 </sst>
 </file>
@@ -671,7 +675,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4070884-C656-4598-9D98-EC54A4CE7753}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.33203125" customWidth="1"/>
@@ -704,7 +708,7 @@
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -716,7 +720,7 @@
       </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -730,9 +734,6 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:4" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>